<commit_message>
Deploying to main from @ open-resource-discovery/specification@b2aad13960c373e050ed1721a025a861eeab48a8 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-218/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-218/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1444" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -376,6 +376,18 @@
     <t>array&lt;ExposedApiResourcesTarget&gt;</t>
   </si>
   <si>
+    <t>relatedCapabilities</t>
+  </si>
+  <si>
+    <t>array&lt;RelatedCapability&gt;</t>
+  </si>
+  <si>
+    <t>relatedAgents</t>
+  </si>
+  <si>
+    <t>array&lt;RelatedAgent&gt;</t>
+  </si>
+  <si>
     <t>integrationDependencies</t>
   </si>
   <si>
@@ -397,12 +409,6 @@
     <t>Capability</t>
   </si>
   <si>
-    <t>relatedCapabilities</t>
-  </si>
-  <si>
-    <t>array&lt;RelatedCapability&gt;</t>
-  </si>
-  <si>
     <t>array&lt;CapabilityDefinition&gt;</t>
   </si>
   <si>
@@ -604,69 +610,12 @@
     <t>correlationId</t>
   </si>
   <si>
-    <t>Generic Relationship</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>RelationshipEndpoint</t>
+    <t>Related Entity Type</t>
   </si>
   <si>
     <t>relationType</t>
   </si>
   <si>
-    <t>target</t>
-  </si>
-  <si>
-    <t>Relationship ORD Endpoint</t>
-  </si>
-  <si>
-    <t>resourceVersion</t>
-  </si>
-  <si>
-    <t>definition</t>
-  </si>
-  <si>
-    <t>RelationshipDefinitionReference</t>
-  </si>
-  <si>
-    <t>element</t>
-  </si>
-  <si>
-    <t>RelationshipElementSelector</t>
-  </si>
-  <si>
-    <t>Relationship External Endpoint</t>
-  </si>
-  <si>
-    <t>uri</t>
-  </si>
-  <si>
-    <t>Relationship Definition Reference</t>
-  </si>
-  <si>
-    <t>sha256</t>
-  </si>
-  <si>
-    <t>Relationship Element By Operation</t>
-  </si>
-  <si>
-    <t>operation</t>
-  </si>
-  <si>
-    <t>Relationship Element By JSON Pointer</t>
-  </si>
-  <si>
-    <t>Relationship Element By Native ID</t>
-  </si>
-  <si>
-    <t>nativeId</t>
-  </si>
-  <si>
-    <t>Related Entity Type</t>
-  </si>
-  <si>
     <t>Related API Resource</t>
   </si>
   <si>
@@ -674,6 +623,9 @@
   </si>
   <si>
     <t>Related Capability</t>
+  </si>
+  <si>
+    <t>Related Agent</t>
   </si>
   <si>
     <t>Exposed Entity Type</t>
@@ -1062,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D495"/>
+  <dimension ref="A1:D481"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4660,7 +4612,7 @@
         <v>0</v>
       </c>
       <c r="D257" t="s">
-        <v>9</v>
+        <v>122</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
@@ -4668,13 +4620,13 @@
         <v>118</v>
       </c>
       <c r="B258" t="s">
-        <v>19</v>
+        <v>123</v>
       </c>
       <c r="C258" t="b">
         <v>0</v>
       </c>
       <c r="D258" t="s">
-        <v>20</v>
+        <v>124</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
@@ -4682,7 +4634,7 @@
         <v>118</v>
       </c>
       <c r="B259" t="s">
-        <v>31</v>
+        <v>125</v>
       </c>
       <c r="C259" t="b">
         <v>0</v>
@@ -4696,13 +4648,13 @@
         <v>118</v>
       </c>
       <c r="B260" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C260" t="b">
         <v>0</v>
       </c>
       <c r="D260" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
@@ -4710,52 +4662,52 @@
         <v>118</v>
       </c>
       <c r="B261" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C261" t="b">
         <v>0</v>
       </c>
       <c r="D261" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B262" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C262" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D262" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B263" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C263" t="b">
         <v>0</v>
       </c>
       <c r="D263" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B264" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C264" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264" t="s">
         <v>6</v>
@@ -4763,13 +4715,13 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B265" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C265" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="s">
         <v>6</v>
@@ -4777,10 +4729,10 @@
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B266" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="C266" t="b">
         <v>0</v>
@@ -4791,10 +4743,10 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B267" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C267" t="b">
         <v>1</v>
@@ -4805,13 +4757,13 @@
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B268" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C268" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D268" t="s">
         <v>6</v>
@@ -4819,108 +4771,108 @@
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B269" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="C269" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B270" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D270" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B271" t="s">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="C271" t="b">
         <v>0</v>
       </c>
       <c r="D271" t="s">
-        <v>123</v>
+        <v>56</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B272" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C272" t="b">
         <v>0</v>
       </c>
       <c r="D272" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B273" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="C273" t="b">
         <v>0</v>
       </c>
       <c r="D273" t="s">
-        <v>33</v>
+        <v>127</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B274" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C274" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D274" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B275" t="s">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="C275" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D275" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B276" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C276" t="b">
         <v>1</v>
@@ -4931,27 +4883,27 @@
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B277" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C277" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D277" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B278" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="C278" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D278" t="s">
         <v>6</v>
@@ -4959,27 +4911,27 @@
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B279" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C279" t="b">
         <v>0</v>
       </c>
       <c r="D279" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B280" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C280" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D280" t="s">
         <v>6</v>
@@ -4987,24 +4939,24 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B281" t="s">
-        <v>8</v>
+        <v>116</v>
       </c>
       <c r="C281" t="b">
         <v>0</v>
       </c>
       <c r="D281" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B282" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C282" t="b">
         <v>1</v>
@@ -5015,27 +4967,27 @@
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B283" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C283" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D283" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B284" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C284" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D284" t="s">
         <v>6</v>
@@ -5043,10 +4995,10 @@
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B285" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C285" t="b">
         <v>1</v>
@@ -5057,10 +5009,10 @@
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B286" t="s">
-        <v>126</v>
+        <v>12</v>
       </c>
       <c r="C286" t="b">
         <v>0</v>
@@ -5071,97 +5023,97 @@
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B287" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C287" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D287" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B288" t="s">
-        <v>32</v>
+        <v>130</v>
       </c>
       <c r="C288" t="b">
         <v>0</v>
       </c>
       <c r="D288" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B289" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C289" t="b">
         <v>0</v>
       </c>
       <c r="D289" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B290" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C290" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D290" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B291" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="C291" t="b">
         <v>0</v>
       </c>
       <c r="D291" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B292" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C292" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D292" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B293" t="s">
-        <v>97</v>
+        <v>7</v>
       </c>
       <c r="C293" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D293" t="s">
         <v>6</v>
@@ -5169,24 +5121,24 @@
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B294" t="s">
-        <v>115</v>
+        <v>8</v>
       </c>
       <c r="C294" t="b">
         <v>0</v>
       </c>
       <c r="D294" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B295" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="C295" t="b">
         <v>1</v>
@@ -5197,10 +5149,10 @@
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B296" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="C296" t="b">
         <v>0</v>
@@ -5211,13 +5163,13 @@
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B297" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C297" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D297" t="s">
         <v>6</v>
@@ -5225,10 +5177,10 @@
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B298" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="C298" t="b">
         <v>0</v>
@@ -5239,13 +5191,13 @@
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B299" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C299" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D299" t="s">
         <v>6</v>
@@ -5253,24 +5205,24 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B300" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C300" t="b">
         <v>0</v>
       </c>
       <c r="D300" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B301" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C301" t="b">
         <v>1</v>
@@ -5281,24 +5233,24 @@
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B302" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C302" t="b">
         <v>0</v>
       </c>
       <c r="D302" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B303" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C303" t="b">
         <v>1</v>
@@ -5309,13 +5261,13 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B304" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C304" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D304" t="s">
         <v>6</v>
@@ -5323,27 +5275,27 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B305" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="C305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D305" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B306" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C306" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D306" t="s">
         <v>6</v>
@@ -5351,142 +5303,142 @@
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B307" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B308" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B309" t="s">
-        <v>57</v>
+        <v>92</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
       </c>
       <c r="D309" t="s">
-        <v>58</v>
+        <v>9</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B310" t="s">
-        <v>128</v>
+        <v>55</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B311" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>130</v>
+        <v>58</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B312" t="s">
-        <v>19</v>
+        <v>121</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B313" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>9</v>
+        <v>132</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B314" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B315" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B316" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
@@ -5494,13 +5446,13 @@
         <v>131</v>
       </c>
       <c r="B317" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="C317" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
@@ -5508,21 +5460,21 @@
         <v>131</v>
       </c>
       <c r="B318" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B319" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C319" t="b">
         <v>1</v>
@@ -5533,13 +5485,13 @@
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B320" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C320" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D320" t="s">
         <v>6</v>
@@ -5547,27 +5499,27 @@
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B321" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C321" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D321" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B322" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="C322" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D322" t="s">
         <v>6</v>
@@ -5575,27 +5527,27 @@
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B323" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B324" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C324" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D324" t="s">
         <v>6</v>
@@ -5603,10 +5555,10 @@
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B325" t="s">
-        <v>7</v>
+        <v>116</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
@@ -5617,27 +5569,27 @@
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B326" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C326" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D326" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B327" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C327" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" t="s">
         <v>6</v>
@@ -5645,27 +5597,27 @@
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B328" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C328" t="b">
         <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B329" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5673,13 +5625,13 @@
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B330" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5687,24 +5639,24 @@
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B331" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C331" t="b">
         <v>0</v>
       </c>
       <c r="D331" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B332" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C332" t="b">
         <v>1</v>
@@ -5715,24 +5667,24 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B333" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C333" t="b">
         <v>0</v>
       </c>
       <c r="D333" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B334" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C334" t="b">
         <v>1</v>
@@ -5743,13 +5695,13 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B335" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="s">
         <v>6</v>
@@ -5757,13 +5709,13 @@
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B336" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="C336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5771,80 +5723,80 @@
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B337" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C337" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D337" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B338" t="s">
-        <v>133</v>
+        <v>60</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B339" t="s">
-        <v>134</v>
+        <v>61</v>
       </c>
       <c r="C339" t="b">
         <v>0</v>
       </c>
       <c r="D339" t="s">
-        <v>135</v>
+        <v>9</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B340" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C340" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D340" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B341" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>20</v>
+        <v>137</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B342" t="s">
-        <v>31</v>
+        <v>138</v>
       </c>
       <c r="C342" t="b">
         <v>0</v>
@@ -5855,304 +5807,304 @@
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B343" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C343" t="b">
         <v>0</v>
       </c>
       <c r="D343" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B344" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C344" t="b">
         <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B345" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C345" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B346" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C346" t="b">
         <v>0</v>
       </c>
       <c r="D346" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B347" t="s">
-        <v>133</v>
+        <v>10</v>
       </c>
       <c r="C347" t="b">
         <v>1</v>
       </c>
       <c r="D347" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B348" t="s">
-        <v>138</v>
+        <v>12</v>
       </c>
       <c r="C348" t="b">
         <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B349" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B350" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B351" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B352" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
+        <v>139</v>
+      </c>
+      <c r="B353" t="s">
         <v>145</v>
       </c>
-      <c r="B353" t="s">
-        <v>5</v>
-      </c>
       <c r="C353" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>6</v>
+        <v>146</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B354" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
       <c r="C354" t="b">
         <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B355" t="s">
-        <v>147</v>
+        <v>5</v>
       </c>
       <c r="C355" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D355" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B356" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
+        <v>147</v>
+      </c>
+      <c r="B357" t="s">
         <v>149</v>
       </c>
-      <c r="B357" t="s">
-        <v>5</v>
-      </c>
       <c r="C357" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B358" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
       <c r="C358" t="b">
         <v>0</v>
       </c>
       <c r="D358" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B359" t="s">
-        <v>147</v>
+        <v>5</v>
       </c>
       <c r="C359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B360" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
+        <v>151</v>
+      </c>
+      <c r="B361" t="s">
         <v>149</v>
       </c>
-      <c r="B361" t="s">
-        <v>32</v>
-      </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>33</v>
+        <v>152</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B362" t="s">
         <v>153</v>
       </c>
       <c r="C362" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B363" t="s">
-        <v>155</v>
+        <v>32</v>
       </c>
       <c r="C363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B364" t="s">
-        <v>5</v>
+        <v>155</v>
       </c>
       <c r="C364" t="b">
         <v>1</v>
@@ -6166,10 +6118,10 @@
         <v>156</v>
       </c>
       <c r="B365" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C365" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D365" t="s">
         <v>6</v>
@@ -6177,27 +6129,27 @@
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B366" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C366" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D366" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B367" t="s">
-        <v>5</v>
+        <v>148</v>
       </c>
       <c r="C367" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D367" t="s">
         <v>6</v>
@@ -6205,72 +6157,72 @@
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B368" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C368" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B369" t="s">
-        <v>158</v>
+        <v>5</v>
       </c>
       <c r="C369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D369" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B370" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C370" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D370" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B371" t="s">
-        <v>32</v>
+        <v>160</v>
       </c>
       <c r="C371" t="b">
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B372" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
@@ -6278,13 +6230,13 @@
         <v>159</v>
       </c>
       <c r="B373" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C373" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
@@ -6292,21 +6244,21 @@
         <v>159</v>
       </c>
       <c r="B374" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="C374" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D374" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B375" t="s">
-        <v>160</v>
+        <v>13</v>
       </c>
       <c r="C375" t="b">
         <v>1</v>
@@ -6317,13 +6269,13 @@
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B376" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="C376" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D376" t="s">
         <v>6</v>
@@ -6331,13 +6283,13 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B377" t="s">
-        <v>99</v>
+        <v>162</v>
       </c>
       <c r="C377" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D377" t="s">
         <v>6</v>
@@ -6348,10 +6300,10 @@
         <v>161</v>
       </c>
       <c r="B378" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" t="s">
         <v>6</v>
@@ -6365,7 +6317,7 @@
         <v>99</v>
       </c>
       <c r="C379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6373,13 +6325,13 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B380" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380" t="s">
         <v>6</v>
@@ -6387,10 +6339,10 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B381" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C381" t="b">
         <v>1</v>
@@ -6401,13 +6353,13 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B382" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
         <v>6</v>
@@ -6415,13 +6367,13 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B383" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6429,10 +6381,10 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B384" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C384" t="b">
         <v>1</v>
@@ -6443,13 +6395,13 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B385" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="s">
         <v>6</v>
@@ -6457,13 +6409,13 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B386" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386" t="s">
         <v>6</v>
@@ -6471,10 +6423,10 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B387" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C387" t="b">
         <v>1</v>
@@ -6485,13 +6437,13 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B388" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="s">
         <v>6</v>
@@ -6499,13 +6451,13 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B389" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C389" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D389" t="s">
         <v>6</v>
@@ -6513,10 +6465,10 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B390" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C390" t="b">
         <v>1</v>
@@ -6527,13 +6479,13 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B391" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" t="s">
         <v>6</v>
@@ -6541,13 +6493,13 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B392" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C392" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D392" t="s">
         <v>6</v>
@@ -6555,10 +6507,10 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B393" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C393" t="b">
         <v>1</v>
@@ -6569,10 +6521,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B394" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="C394" t="b">
         <v>0</v>
@@ -6583,13 +6535,13 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B395" t="s">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="C395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D395" t="s">
         <v>6</v>
@@ -6597,58 +6549,58 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B396" t="s">
-        <v>8</v>
+        <v>169</v>
       </c>
       <c r="C396" t="b">
         <v>0</v>
       </c>
       <c r="D396" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B397" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B398" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C398" t="b">
         <v>0</v>
       </c>
       <c r="D398" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B399" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
       </c>
       <c r="D399" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
@@ -6656,13 +6608,13 @@
         <v>168</v>
       </c>
       <c r="B400" t="s">
-        <v>169</v>
+        <v>34</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
@@ -6670,7 +6622,7 @@
         <v>168</v>
       </c>
       <c r="B401" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C401" t="b">
         <v>0</v>
@@ -6681,44 +6633,44 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B402" t="s">
-        <v>32</v>
+        <v>171</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
       </c>
       <c r="D402" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B403" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B404" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C404" t="b">
         <v>0</v>
       </c>
       <c r="D404" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
@@ -6726,13 +6678,13 @@
         <v>170</v>
       </c>
       <c r="B405" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
@@ -6740,108 +6692,108 @@
         <v>170</v>
       </c>
       <c r="B406" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B407" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B408" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B409" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B410" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B411" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="C411" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B412" t="s">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>172</v>
+        <v>97</v>
       </c>
       <c r="C413" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D413" t="s">
         <v>6</v>
@@ -6852,10 +6804,10 @@
         <v>173</v>
       </c>
       <c r="B414" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C414" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D414" t="s">
         <v>6</v>
@@ -6866,7 +6818,7 @@
         <v>173</v>
       </c>
       <c r="B415" t="s">
-        <v>115</v>
+        <v>174</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
@@ -6877,13 +6829,13 @@
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B416" t="s">
-        <v>172</v>
+        <v>97</v>
       </c>
       <c r="C416" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D416" t="s">
         <v>6</v>
@@ -6891,10 +6843,10 @@
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B417" t="s">
-        <v>174</v>
+        <v>115</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
@@ -6908,10 +6860,10 @@
         <v>175</v>
       </c>
       <c r="B418" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C418" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D418" t="s">
         <v>6</v>
@@ -6922,10 +6874,10 @@
         <v>175</v>
       </c>
       <c r="B419" t="s">
-        <v>10</v>
+        <v>176</v>
       </c>
       <c r="C419" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6933,13 +6885,13 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B420" t="s">
-        <v>12</v>
+        <v>178</v>
       </c>
       <c r="C420" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D420" t="s">
         <v>6</v>
@@ -6947,83 +6899,83 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B421" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C421" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D421" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B422" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B423" t="s">
-        <v>177</v>
+        <v>32</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B424" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B425" t="s">
         <v>179</v>
       </c>
       <c r="C425" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B426" t="s">
-        <v>176</v>
+        <v>38</v>
       </c>
       <c r="C426" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D426" t="s">
         <v>6</v>
@@ -7031,10 +6983,10 @@
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B427" t="s">
-        <v>10</v>
+        <v>181</v>
       </c>
       <c r="C427" t="b">
         <v>1</v>
@@ -7045,13 +6997,13 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
+        <v>180</v>
+      </c>
+      <c r="B428" t="s">
         <v>178</v>
       </c>
-      <c r="B428" t="s">
-        <v>12</v>
-      </c>
       <c r="C428" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D428" t="s">
         <v>6</v>
@@ -7059,80 +7011,80 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B429" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D429" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B430" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
       </c>
       <c r="D430" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B431" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
       </c>
       <c r="D431" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B432" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
       </c>
       <c r="D432" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>84</v>
+        <v>180</v>
       </c>
       <c r="B433" t="s">
-        <v>180</v>
+        <v>46</v>
       </c>
       <c r="C433" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>84</v>
+        <v>180</v>
       </c>
       <c r="B434" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
@@ -7143,58 +7095,58 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>181</v>
+        <v>84</v>
       </c>
       <c r="B435" t="s">
         <v>182</v>
       </c>
       <c r="C435" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D435" t="s">
-        <v>183</v>
+        <v>6</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>181</v>
+        <v>84</v>
       </c>
       <c r="B436" t="s">
-        <v>184</v>
+        <v>12</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>185</v>
+        <v>6</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B437" t="s">
-        <v>5</v>
+        <v>184</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
-        <v>6</v>
+        <v>185</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
+        <v>183</v>
+      </c>
+      <c r="B438" t="s">
         <v>186</v>
       </c>
-      <c r="B438" t="s">
+      <c r="C438" t="b">
+        <v>1</v>
+      </c>
+      <c r="D438" t="s">
         <v>187</v>
-      </c>
-      <c r="C438" t="b">
-        <v>1</v>
-      </c>
-      <c r="D438" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
@@ -7216,7 +7168,7 @@
         <v>188</v>
       </c>
       <c r="B440" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C440" t="b">
         <v>1</v>
@@ -7227,10 +7179,10 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B441" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="C441" t="b">
         <v>1</v>
@@ -7241,10 +7193,10 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
+        <v>190</v>
+      </c>
+      <c r="B442" t="s">
         <v>189</v>
-      </c>
-      <c r="B442" t="s">
-        <v>190</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7286,7 +7238,7 @@
         <v>193</v>
       </c>
       <c r="B445" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7297,10 +7249,10 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
+        <v>193</v>
+      </c>
+      <c r="B446" t="s">
         <v>194</v>
-      </c>
-      <c r="B446" t="s">
-        <v>5</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7314,7 +7266,7 @@
         <v>195</v>
       </c>
       <c r="B447" t="s">
-        <v>196</v>
+        <v>5</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7325,10 +7277,10 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B448" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C448" t="b">
         <v>1</v>
@@ -7348,15 +7300,15 @@
         <v>1</v>
       </c>
       <c r="D449" t="s">
-        <v>199</v>
+        <v>6</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B450" t="s">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
@@ -7367,24 +7319,24 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B451" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="s">
-        <v>199</v>
+        <v>6</v>
       </c>
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B452" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C452" t="b">
         <v>1</v>
@@ -7395,10 +7347,10 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B453" t="s">
-        <v>12</v>
+        <v>200</v>
       </c>
       <c r="C453" t="b">
         <v>0</v>
@@ -7409,16 +7361,16 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B454" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C454" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D454" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
@@ -7426,10 +7378,10 @@
         <v>202</v>
       </c>
       <c r="B455" t="s">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="C455" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D455" t="s">
         <v>6</v>
@@ -7437,13 +7389,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B456" t="s">
-        <v>203</v>
+        <v>5</v>
       </c>
       <c r="C456" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7451,41 +7403,41 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B457" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C457" t="b">
         <v>0</v>
       </c>
       <c r="D457" t="s">
-        <v>205</v>
+        <v>6</v>
       </c>
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B458" t="s">
-        <v>206</v>
+        <v>5</v>
       </c>
       <c r="C458" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D458" t="s">
-        <v>207</v>
+        <v>6</v>
       </c>
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B459" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="C459" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7493,10 +7445,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B460" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7507,13 +7459,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B461" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="C461" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7521,10 +7473,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B462" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
       <c r="C462" t="b">
         <v>0</v>
@@ -7535,13 +7487,13 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B463" t="s">
-        <v>213</v>
+        <v>178</v>
       </c>
       <c r="C463" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7549,10 +7501,10 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B464" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C464" t="b">
         <v>1</v>
@@ -7563,13 +7515,13 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B465" t="s">
-        <v>216</v>
+        <v>12</v>
       </c>
       <c r="C465" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D465" t="s">
         <v>6</v>
@@ -7577,7 +7529,7 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B466" t="s">
         <v>5</v>
@@ -7591,10 +7543,10 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="B467" t="s">
-        <v>200</v>
+        <v>7</v>
       </c>
       <c r="C467" t="b">
         <v>0</v>
@@ -7605,27 +7557,27 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="B468" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="B469" t="s">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7633,13 +7585,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="B470" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7647,13 +7599,13 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="B471" t="s">
-        <v>200</v>
+        <v>12</v>
       </c>
       <c r="C471" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7661,10 +7613,10 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="B472" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="C472" t="b">
         <v>1</v>
@@ -7675,24 +7627,24 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="C473" t="b">
         <v>0</v>
       </c>
       <c r="D473" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="B474" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C474" t="b">
         <v>1</v>
@@ -7703,10 +7655,10 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="B475" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C475" t="b">
         <v>0</v>
@@ -7717,13 +7669,13 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>179</v>
+        <v>38</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7731,13 +7683,13 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>176</v>
+        <v>52</v>
       </c>
       <c r="C477" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D477" t="s">
         <v>6</v>
@@ -7745,253 +7697,57 @@
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="B478" t="s">
-        <v>223</v>
+        <v>19</v>
       </c>
       <c r="C478" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D478" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="B479" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
       </c>
       <c r="D479" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="B480" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C480" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D480" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="B481" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="C481" t="b">
         <v>0</v>
       </c>
       <c r="D481" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A482" t="s">
-        <v>224</v>
-      </c>
-      <c r="B482" t="s">
-        <v>8</v>
-      </c>
-      <c r="C482" t="b">
-        <v>0</v>
-      </c>
-      <c r="D482" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A483" t="s">
-        <v>224</v>
-      </c>
-      <c r="B483" t="s">
-        <v>10</v>
-      </c>
-      <c r="C483" t="b">
-        <v>1</v>
-      </c>
-      <c r="D483" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A484" t="s">
-        <v>224</v>
-      </c>
-      <c r="B484" t="s">
-        <v>11</v>
-      </c>
-      <c r="C484" t="b">
-        <v>0</v>
-      </c>
-      <c r="D484" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A485" t="s">
-        <v>224</v>
-      </c>
-      <c r="B485" t="s">
-        <v>12</v>
-      </c>
-      <c r="C485" t="b">
-        <v>1</v>
-      </c>
-      <c r="D485" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A486" t="s">
-        <v>224</v>
-      </c>
-      <c r="B486" t="s">
-        <v>45</v>
-      </c>
-      <c r="C486" t="b">
-        <v>1</v>
-      </c>
-      <c r="D486" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A487" t="s">
-        <v>224</v>
-      </c>
-      <c r="B487" t="s">
-        <v>46</v>
-      </c>
-      <c r="C487" t="b">
-        <v>0</v>
-      </c>
-      <c r="D487" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A488" t="s">
-        <v>224</v>
-      </c>
-      <c r="B488" t="s">
-        <v>13</v>
-      </c>
-      <c r="C488" t="b">
-        <v>1</v>
-      </c>
-      <c r="D488" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A489" t="s">
-        <v>224</v>
-      </c>
-      <c r="B489" t="s">
-        <v>37</v>
-      </c>
-      <c r="C489" t="b">
-        <v>0</v>
-      </c>
-      <c r="D489" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A490" t="s">
-        <v>224</v>
-      </c>
-      <c r="B490" t="s">
-        <v>38</v>
-      </c>
-      <c r="C490" t="b">
-        <v>1</v>
-      </c>
-      <c r="D490" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A491" t="s">
-        <v>224</v>
-      </c>
-      <c r="B491" t="s">
-        <v>52</v>
-      </c>
-      <c r="C491" t="b">
-        <v>1</v>
-      </c>
-      <c r="D491" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A492" t="s">
-        <v>224</v>
-      </c>
-      <c r="B492" t="s">
-        <v>19</v>
-      </c>
-      <c r="C492" t="b">
-        <v>0</v>
-      </c>
-      <c r="D492" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A493" t="s">
-        <v>224</v>
-      </c>
-      <c r="B493" t="s">
-        <v>31</v>
-      </c>
-      <c r="C493" t="b">
-        <v>0</v>
-      </c>
-      <c r="D493" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A494" t="s">
-        <v>224</v>
-      </c>
-      <c r="B494" t="s">
-        <v>32</v>
-      </c>
-      <c r="C494" t="b">
-        <v>0</v>
-      </c>
-      <c r="D494" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="495" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A495" t="s">
-        <v>224</v>
-      </c>
-      <c r="B495" t="s">
-        <v>34</v>
-      </c>
-      <c r="C495" t="b">
-        <v>0</v>
-      </c>
-      <c r="D495" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>